<commit_message>
Epic 7 tracker: sync CRM + Team/People work shipped this sprint
Standing rule: tracker updates land side-by-side with code, not batched.

Marked Done:
- U7-07.2 (ContactProfile 360 density) -- eeca877
- U7-07.5 (Contact card unified shape) -- eeca877
- U7-10.1 (Team vs People clarify)     -- b7cd6ee + 349a7b4 + f8c13ea

Added:
- U7-07.7  CRM scope simplified to Buyers|Suppliers only  (a1498ed)
- U7-07.8  Add-contact menu + dialog polish               (e08f5ae)
- U7-10.6  Team page HRM redesign + attendance killed     (349a7b4)

Dashboard: 26/138 (18.8%) -> 32/141 (22.7%).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
@@ -1472,7 +1472,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 7 progress: 26 of 138 items Done  (18.8%)</t>
+          <t>Epic 7 progress: 32 of 141 items Done  (22.7%)</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L139"/>
+  <dimension ref="A1:L142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5290,11 +5290,15 @@
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J59" s="16" t="inlineStr"/>
-      <c r="K59" s="16" t="inlineStr"/>
+      <c r="K59" s="16" t="inlineStr">
+        <is>
+          <t>Shipped 2026-08-17 (commit eeca877 -- CRM Batch 2). Killed 6 "nothing here" placeholder sections via new hideWhenEmpty prop on Section. AI Relationship Intelligence card collapsed to a compact inline prompt when unscored (was a huge empty card). Deduped invoices/payments/complaints/workflows by id so the backend duplicate-return no longer double-renders. "Back to People" -&gt; "Back to CRM" now routes to /crm.</t>
+        </is>
+      </c>
       <c r="L59" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5446,11 +5450,15 @@
       </c>
       <c r="I62" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J62" s="18" t="inlineStr"/>
-      <c r="K62" s="18" t="inlineStr"/>
+      <c r="K62" s="18" t="inlineStr">
+        <is>
+          <t>Shipped 2026-08-17 (commit eeca877 -- CRM Batch 1). Card density fixed: 11+ elements per card collapsed to 5 (name + status dot + one type chip + lifecycle chip + one key signal + touched-ago). Chips use tenant lexicon (L.customer_singular / L.vendor_singular) so BUYER/SUPPLIER match everywhere. Whole card is click-target -- redundant per-card 360deg icon killed.</t>
+        </is>
+      </c>
       <c r="L62" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6174,11 +6182,15 @@
       </c>
       <c r="I76" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J76" s="18" t="inlineStr"/>
-      <c r="K76" s="18" t="inlineStr"/>
+      <c r="K76" s="18" t="inlineStr">
+        <is>
+          <t>Shipped 2026-08-17 (commits b7cd6ee + 349a7b4 + this push -- U7-09.TEAM/PEOPLE). Team is now a viewable-by-all HRM roster with click-through profile dialog and no attendance concerns (killed the attendance-portal framing). People became a three-tab admin page (Employees / Customers / Vendors) with per-tab edit gating: team_manage for Employees, "people" perm for Customers+Vendors. Every user sees the roster; owner + perm-holders keep edit affordances.</t>
+        </is>
+      </c>
       <c r="L76" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -9594,6 +9606,174 @@
       <c r="L139" s="16" t="inlineStr">
         <is>
           <t>Own audit 2026-08-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="70" customHeight="1">
+      <c r="A140" s="16" t="inlineStr">
+        <is>
+          <t>U7-07.7</t>
+        </is>
+      </c>
+      <c r="B140" s="16" t="inlineStr">
+        <is>
+          <t>CRM.js, Contacts.js, ContactProfile.js</t>
+        </is>
+      </c>
+      <c r="C140" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="D140" s="15" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="E140" s="16" t="inlineStr">
+        <is>
+          <t>CRM scope simplified to Buyers | Suppliers only</t>
+        </is>
+      </c>
+      <c r="F140" s="16" t="inlineStr">
+        <is>
+          <t>Old header carried 5 chips: All / Customers / Suppliers / Mine / With complaints. Founder ask: each user works in one lane at a time; complaints are already visible via the red pill on every card (Batch 1) so a dedicated tab is redundant. Reduce to two big HRM-style segmented tabs -- Buyers | Suppliers -- with count badges; move search/status/sort to a subtler filter strip below the tabs.</t>
+        </is>
+      </c>
+      <c r="G140" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H140" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I140" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J140" s="16" t="n"/>
+      <c r="K140" s="16" t="inlineStr">
+        <is>
+          <t>Shipped 2026-08-17 (commit a1498ed). SCOPES trimmed from 5 to 2. Killed the useEffect that force-flipped scope to "complaints" on ?complaint=open deep-link (Desk Trends still lands on Buyers; users spot the red pills). Default scope = customers.</t>
+        </is>
+      </c>
+      <c r="L140" s="16" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-08-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="70" customHeight="1">
+      <c r="A141" s="16" t="inlineStr">
+        <is>
+          <t>U7-07.8</t>
+        </is>
+      </c>
+      <c r="B141" s="16" t="inlineStr">
+        <is>
+          <t>CRM.js, Contacts.js, ContactProfile.js</t>
+        </is>
+      </c>
+      <c r="C141" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="D141" s="15" t="inlineStr">
+        <is>
+          <t>Interaction</t>
+        </is>
+      </c>
+      <c r="E141" s="16" t="inlineStr">
+        <is>
+          <t>Add-contact flow -- menu + dialog polish</t>
+        </is>
+      </c>
+      <c r="F141" s="16" t="inlineStr">
+        <is>
+          <t>Header dropdown was &lt;details&gt;/&lt;summary&gt; with cramped label-mono subtitles that read as jumbled uppercase labels ("BUYER / RETAIL, ACCOUNT / DEALER"). Dialog behind it was 10 fields dumped into a 2-col grid with no hierarchy. Rebuild: controlled menu with a Phosphor icon per option, wider (300px), normal-case helper text, backdrop click + Escape to close. Dialog: segmented CUSTOMER/DEALER/SUPPLIER tabs, auto-focused name, sectioned layout (Identity / Contact / Classification), advanced fields (GSTIN, address, tags, owner, notes) collapsed behind "More details" toggle.</t>
+        </is>
+      </c>
+      <c r="G141" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H141" s="16" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I141" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J141" s="16" t="n"/>
+      <c r="K141" s="16" t="inlineStr">
+        <is>
+          <t>Shipped 2026-08-17 (this push). Backdrop pattern (not document.mousedown) avoids a race with React 18 Strict Mode dev-only double-invocation that was closing the menu on the same click that opened it. Advanced section auto-expands when editing an existing contact so nothing looks missing.</t>
+        </is>
+      </c>
+      <c r="L141" s="16" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-08-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="70" customHeight="1">
+      <c r="A142" s="16" t="inlineStr">
+        <is>
+          <t>U7-10.6</t>
+        </is>
+      </c>
+      <c r="B142" s="16" t="inlineStr">
+        <is>
+          <t>Team.js, People.js, WorkCoach.js</t>
+        </is>
+      </c>
+      <c r="C142" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="D142" s="15" t="inlineStr">
+        <is>
+          <t>Visual</t>
+        </is>
+      </c>
+      <c r="E142" s="16" t="inlineStr">
+        <is>
+          <t>Team page redesign -- HRM roster + click-through profile</t>
+        </is>
+      </c>
+      <c r="F142" s="16" t="inlineStr">
+        <is>
+          <t>Team page read as an attendance portal (present/absent chips, day toggle, roster as a flat list). Founder ask: this is not attendance; make it feel like an HRM tool. Killed attendance entirely (removed /attendance useQuery + toggleAbsent). Roster is now a card grid grouped by role, with a subtle status dot (active green / pending amber / suspended gray) sourced from invite_status. Clicking a card opens a profile dialog carrying contact info + access controls -- access moved INSIDE the card so perm-holders can grant/edit from there.</t>
+        </is>
+      </c>
+      <c r="G142" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H142" s="16" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="I142" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J142" s="16" t="n"/>
+      <c r="K142" s="16" t="inlineStr">
+        <is>
+          <t>Shipped 2026-08-17 (commit 349a7b4). Everyone sees the roster (perm gate dropped in App.js -- &lt;Protected&gt; replaces &lt;Protected perms={{team_manage}}&gt;). Non-perm-holders see the roster read-only; team_manage/owner see edit affordances.</t>
+        </is>
+      </c>
+      <c r="L142" s="16" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-08-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
U7-05.10: rename MyWork view toggle "My Work" -> "Tasks" (kill dup)
Owner ask: "In the owner access of work section, my we are showing
my work 2 times". Desktop MyWork toolbar had a view toggle labeled
MY WORK sitting next to WORKFLOWS and LEAVE, but the page itself is
also "My Work" (sidebar nav entry). Two identical labels on one
viewport.

Rename the toggle to TASKS across en/hi/ta. Trio now reads
TASKS / WORKFLOWS / LEAVE. Mobile MyWorkMobile already used
"Tasks" for this toggle -- desktop was the outlier.

Only the label changes; view_mywork translation key stays put so
no call sites need updating.

Tracker: 32/141 -> 33/142.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
@@ -1472,7 +1472,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 7 progress: 32 of 141 items Done  (22.7%)</t>
+          <t>Epic 7 progress: 33 of 142 items Done  (23.2%)</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L142"/>
+  <dimension ref="A1:L143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -9777,6 +9777,62 @@
         </is>
       </c>
     </row>
+    <row r="143" ht="70" customHeight="1">
+      <c r="A143" s="18" t="inlineStr">
+        <is>
+          <t>U7-05.10</t>
+        </is>
+      </c>
+      <c r="B143" s="18" t="inlineStr">
+        <is>
+          <t>MyWork.js, i18n.js</t>
+        </is>
+      </c>
+      <c r="C143" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D143" s="17" t="inlineStr">
+        <is>
+          <t>Copy</t>
+        </is>
+      </c>
+      <c r="E143" s="18" t="inlineStr">
+        <is>
+          <t>MyWork view toggle -- "My Work" duplicates the page title</t>
+        </is>
+      </c>
+      <c r="F143" s="18" t="inlineStr">
+        <is>
+          <t>The desktop MyWork toolbar had a view toggle labeled "MY WORK" that sat next to WORKFLOWS and LEAVE. But the page itself is also called "My Work" (sidebar nav + PageHeader eyebrow/title). Owner ask: "In the owner access of work section, my we are showing my work 2 times". Rename the view toggle to TASKS across en/hi/ta so the trio reads TASKS / WORKFLOWS / LEAVE and the page-title "My Work" only appears once in the viewport. Mobile MyWorkMobile already used "Tasks" for this toggle -- desktop was the outlier.</t>
+        </is>
+      </c>
+      <c r="G143" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H143" s="18" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I143" s="23" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J143" s="18" t="n"/>
+      <c r="K143" s="18" t="inlineStr">
+        <is>
+          <t>Shipped 2026-08-17 (single-line i18n change). Only the view-toggle label changes; view_mywork translation key kept for compatibility.</t>
+        </is>
+      </c>
+      <c r="L143" s="18" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-08-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
U7-08.2: remove Fix Old Purchases button from Finance header
Owner ask: "remove the Fix old purchases button". The button ran
/ledger/reclassify-purchases -- an AI re-classification pass on
historical purchase bills. Every new capture is already classified
at ingest, so the manual re-run has become admin tooling, not
day-to-day owner workflow.

Removed the button + its useState + handler from Ledger.js. Mobile
keeps its own affordance ("Recheck earlier bills" in
FinanceMobile.jsx §8) and the /ledger/reclassify-purchases endpoint
stays live so an admin can trigger it if needed.

Tracker: 36/145 -> 37/146 Done (25.3%).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
@@ -1472,7 +1472,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 7 progress: 36 of 145 items Done  (24.8%)</t>
+          <t>Epic 7 progress: 37 of 146 items Done  (25.3%)</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L146"/>
+  <dimension ref="A1:L147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10001,6 +10001,62 @@
         </is>
       </c>
     </row>
+    <row r="147" ht="70" customHeight="1">
+      <c r="A147" s="18" t="inlineStr">
+        <is>
+          <t>U7-08.2</t>
+        </is>
+      </c>
+      <c r="B147" s="18" t="inlineStr">
+        <is>
+          <t>Ledger.js</t>
+        </is>
+      </c>
+      <c r="C147" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="D147" s="17" t="inlineStr">
+        <is>
+          <t>IA</t>
+        </is>
+      </c>
+      <c r="E147" s="18" t="inlineStr">
+        <is>
+          <t>Remove Fix Old Purchases button from Finance header</t>
+        </is>
+      </c>
+      <c r="F147" s="18" t="inlineStr">
+        <is>
+          <t>Owner ask: "remove the Fix old purchases button". The button ran /ledger/reclassify-purchases -- an AI re-classification pass on historical purchase bills. The new capture pipeline already runs classification on every bill at ingest, so the manual re-run has become admin tooling, not day-to-day owner workflow. Removed the button + its useState + handler from Ledger.js. Mobile keeps its own affordance ("Recheck earlier bills" in FinanceMobile.jsx) and the /ledger/reclassify-purchases endpoint stays live so an admin can trigger it if needed.</t>
+        </is>
+      </c>
+      <c r="G147" s="18" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H147" s="18" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I147" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J147" s="18" t="n"/>
+      <c r="K147" s="18" t="inlineStr">
+        <is>
+          <t>Shipped 2026-08-17. Verified: desktop Finance header now reads OVERVIEW  REVENUE  EXPENSES  ASSETS  INVENTORY  INBOX  + ADD INCOME -- no Fix Old Purchases button.</t>
+        </is>
+      </c>
+      <c r="L147" s="18" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-08-17</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Epic 7 tracker: backfill RD-6 + RD-6.1 rows
Readability/density pass (2b6ab57) and the Desk width fix (f8523ba)
shipped last session without a tracker update -- standing rule is
side-by-side, no exceptions. Logged both now before using the tracker
as the source of truth for the client quotation.

Tracker: 50/160 -> 52/162 Done (32.1%).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
@@ -1472,7 +1472,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 7 progress: 50 of 160 items Done  (31.2%)</t>
+          <t>Epic 7 progress: 52 of 162 items Done  (32.1%)</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L161"/>
+  <dimension ref="A1:L163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -10841,6 +10841,118 @@
         </is>
       </c>
     </row>
+    <row r="162" ht="70" customHeight="1">
+      <c r="A162" s="16" t="inlineStr">
+        <is>
+          <t>RD-6</t>
+        </is>
+      </c>
+      <c r="B162" s="16" t="inlineStr">
+        <is>
+          <t>tailwind.config.js, index.css, Layout.js, 22 pages/components</t>
+        </is>
+      </c>
+      <c r="C162" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="D162" s="15" t="inlineStr">
+        <is>
+          <t>Design system</t>
+        </is>
+      </c>
+      <c r="E162" s="16" t="inlineStr">
+        <is>
+          <t>Readability + density pass -- type scale, sidebar, whitespace</t>
+        </is>
+      </c>
+      <c r="F162" s="16" t="inlineStr">
+        <is>
+          <t>Founder: "its not readable, side bar is small, fonts are small ... there is lot of white space there also ... give me the premium look." Measured before touching anything: 424 text-sm (14px) + 322 text-xs (12px) call sites against only 36 text-base -- almost every word in the app was 12-14px. Fixed via one Tailwind fontSize override (xs 12-&gt;13, sm 14-&gt;15, lg 18-&gt;19, xl 20-&gt;22, 2xl 24-&gt;27, 3xl 30-&gt;34, 4xl 36-&gt;42) so all 746 call sites lifted without per-site edits, plus killed 104 hardcoded text-[9/10/11px] literals that bypassed the scale. Sidebar: the 58px icon-only rail from RD-1 (names visible only on hover) replaced with a 240px labelled sidebar -- always-visible 15px labels, 40px rows, the wordmark restored to its top-left cell, user block showing name + workspace. Whitespace: py-20/16 -&gt; py-12, mb-10/8 -&gt; mb-6, mt-8 -&gt; mt-6, gap-8 -&gt; gap-6, p-12/10 -&gt; p-8 across 22 files.</t>
+        </is>
+      </c>
+      <c r="G162" s="16" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="H162" s="16" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="I162" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J162" s="16" t="n"/>
+      <c r="K162" s="16" t="inlineStr">
+        <is>
+          <t>Shipped 2026-08-18 (commit 2b6ab57). TWO BUGS found and fixed, both making desktop render SMALLER type than mobile: (1) .label-mono had competing definitions -- @apply text-xs but a later rule set font-size: var(--text-label), which was 11px on desktop / 13px on mobile, so every eyebrow painted at 11px regardless of the utility; (2) the Recharts font-size override lived inside the mobile-only media query, so every chart axis was 11px on desktop / 13px on mobile. Also consolidated a second competing accent (brand-blue #002FA7 sitting beside the indigo primary #373ACD) onto the semantic ramp across 37 call sites, and fixed ACTIVITY_META in ContactProfile which had escaped every earlier sweep and still carried bg-brand-green -- the same phantom undefined token found on the CRM lifecycle chip. Verified by measuring the painted font-size of every leaf text node on 9 screens: zero sub-13px text anywhere.</t>
+        </is>
+      </c>
+      <c r="L162" s="16" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="70" customHeight="1">
+      <c r="A163" s="16" t="inlineStr">
+        <is>
+          <t>RD-6.1</t>
+        </is>
+      </c>
+      <c r="B163" s="16" t="inlineStr">
+        <is>
+          <t>Desk.js</t>
+        </is>
+      </c>
+      <c r="C163" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="D163" s="15" t="inlineStr">
+        <is>
+          <t>Design system</t>
+        </is>
+      </c>
+      <c r="E163" s="16" t="inlineStr">
+        <is>
+          <t>Widen Desk content column; fix a JSX comment bug</t>
+        </is>
+      </c>
+      <c r="F163" s="16" t="inlineStr">
+        <is>
+          <t>Desk was capped at max-w-5xl (1024px). With the 240px sidebar already taking width that left ~90px dead either side at 1440px and ~330px at 1920px -- part of the "lot of white space" complaint. Widened to max-w-6xl (1136px).</t>
+        </is>
+      </c>
+      <c r="G163" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H163" s="16" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="I163" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J163" s="16" t="n"/>
+      <c r="K163" s="16" t="inlineStr">
+        <is>
+          <t>Shipped 2026-08-18 (commit f8523ba). Self-caught process bug: the first attempt wrote the explanatory comment as {{/* ... */}} directly inside return (, making it a sibling of the root element -- invalid JSX. The dev server kept serving the previous bundle, so the change looked like a no-op (DOM still reported max-w-5xl while the file on disk said 6xl). Fixed by moving the comment above the return as a plain // comment, then audited the rest of the session for the same pattern and parse-checked the entire tree through @babel/preset-react -- 155 files, all clean. Verified live: every screen now uses ~95% of its content column width.</t>
+        </is>
+      </c>
+      <c r="L163" s="16" t="inlineStr">
+        <is>
+          <t>Founder ask 2026-08-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Epic 7: validate backlog against merged karma UI (2026-08-20)
Screen-by-screen validation of all 110 open Epic 7 items against the
new karma redesign now on Backend_optimization:
- 14 marked Done (already implemented by the redesign)
- 7 Dropped as obsolete (Contacts/CRM merged, FinanceMobile/TeamMobile
  retired for responsive pages, Desk chip-row replaced by DecisionBento,
  board-vs-list settled, owner-gate superseded, signup wizard removed)
- 41 re-scoped to Partial and 48 kept as real blockers, each with dated
  code evidence in Notes.

Operating Score backend batch (U7-01.27-39) confirmed still open.
Recomputed dashboards: Epic 7 = 64/153 in-scope Done (42%);
all-epics = 249/367 (68%).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
@@ -1443,7 +1443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1472,7 +1472,7 @@
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
         <is>
-          <t>Epic 7 progress: 50 of 160 items Done  (31.2%)</t>
+          <t>Epic 7 progress: 64 of 153 in-scope items Done  (42%).  7 items dropped as obsolete after the karma redesign; validated screen-by-screen vs the new UI on 2026-08-20.</t>
         </is>
       </c>
     </row>
@@ -1525,14 +1525,14 @@
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D6" s="12" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E6" s="12" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>51%</t>
         </is>
       </c>
       <c r="F6" s="14" t="inlineStr">
@@ -1558,19 +1558,19 @@
         </is>
       </c>
       <c r="C7" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>40%</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G7" s="16" t="inlineStr">
@@ -1591,19 +1591,19 @@
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D8" s="17" t="n">
         <v>7</v>
       </c>
       <c r="E8" s="17" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="F8" s="17" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G8" s="18" t="inlineStr">
@@ -1627,7 +1627,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
@@ -1690,19 +1690,19 @@
         </is>
       </c>
       <c r="C11" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D11" s="15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>20%</t>
         </is>
       </c>
       <c r="F11" s="15" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G11" s="16" t="inlineStr">
@@ -1723,19 +1723,19 @@
         </is>
       </c>
       <c r="C12" s="17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D12" s="17" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E12" s="17" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G12" s="18" t="inlineStr">
@@ -1759,7 +1759,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="15" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
@@ -1822,19 +1822,19 @@
         </is>
       </c>
       <c r="C15" s="15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D15" s="15" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="F15" s="15" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G15" s="16" t="inlineStr">
@@ -2020,19 +2020,19 @@
         </is>
       </c>
       <c r="C21" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D21" s="15" t="n">
         <v>6</v>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>33%</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G21" s="16" t="inlineStr">
@@ -2053,19 +2053,19 @@
         </is>
       </c>
       <c r="C22" s="17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D22" s="17" t="n">
         <v>5</v>
       </c>
       <c r="E22" s="17" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>60%</t>
         </is>
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="G22" s="18" t="inlineStr">
@@ -2104,6 +2104,39 @@
       <c r="G23" s="16" t="inlineStr">
         <is>
           <t>UX copy sweep (buttons, empty states, errors, tooltips). Final E2E golden path across desktop + mobile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Redesign log</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>KR/RD redesign changelog (shipped during rebuild)</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>21</v>
+      </c>
+      <c r="D24" t="n">
+        <v>22</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Items logged during the karma/KR redesign + RD token retune; filed under Sprint 7 in the backlog. Mostly already shipped.</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2331,11 @@
         </is>
       </c>
       <c r="J3" s="13" t="inlineStr"/>
-      <c r="K3" s="13" t="inlineStr"/>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Score numeral counts up (CountUp, reduced-motion guarded); ArcGauge ring fill doesn't animate from 0 on mount.</t>
+        </is>
+      </c>
       <c r="L3" s="13" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -2854,7 +2891,11 @@
         </is>
       </c>
       <c r="J13" s="13" t="inlineStr"/>
-      <c r="K13" s="13" t="inlineStr"/>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No hover WorkCoach mini-card on leaderboard rows.</t>
+        </is>
+      </c>
       <c r="L13" s="13" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3182,11 +3223,15 @@
       </c>
       <c r="I19" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J19" s="13" t="inlineStr"/>
-      <c r="K19" s="13" t="inlineStr"/>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: Page rewritten on karma semantic tokens; 0 pre-rebrand hardcoded colors (OperatingScore.js).</t>
+        </is>
+      </c>
       <c r="L19" s="13" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3234,11 +3279,15 @@
       </c>
       <c r="I20" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J20" s="13" t="inlineStr"/>
-      <c r="K20" s="13" t="inlineStr"/>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: Adopted DS type ramp font-display + text-h2/h3; only intended font-mono numerals remain.</t>
+        </is>
+      </c>
       <c r="L20" s="13" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3346,7 +3395,11 @@
         </is>
       </c>
       <c r="J22" s="13" t="inlineStr"/>
-      <c r="K22" s="13" t="inlineStr"/>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: ScoreMeter role=progressbar + values added; per-category descriptive aria-label + overall progressbar still missing.</t>
+        </is>
+      </c>
       <c r="L22" s="13" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3398,7 +3451,11 @@
         </is>
       </c>
       <c r="J23" s="13" t="inlineStr"/>
-      <c r="K23" s="13" t="inlineStr"/>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No OperatingScoreMobile / responsive mobile pass (also U7-17.1).</t>
+        </is>
+      </c>
       <c r="L23" s="13" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3446,11 +3503,15 @@
       </c>
       <c r="I24" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="J24" s="13" t="inlineStr"/>
-      <c r="K24" s="13" t="inlineStr"/>
+      <c r="K24" s="13" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DROP: Superseded by Phase A: owner-only gate removed, non-owners get real SelfView, nav shown to all; 403 gone (server.py:2892).</t>
+        </is>
+      </c>
       <c r="L24" s="13" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3502,7 +3563,11 @@
         </is>
       </c>
       <c r="J25" s="13" t="inlineStr"/>
-      <c r="K25" s="13" t="inlineStr"/>
+      <c r="K25" s="13" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Weekly ops-score email opt-in toggle + template not built (frontend of U7-01.38).</t>
+        </is>
+      </c>
       <c r="L25" s="13" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3554,7 +3619,11 @@
         </is>
       </c>
       <c r="J26" s="13" t="inlineStr"/>
-      <c r="K26" s="13" t="inlineStr"/>
+      <c r="K26" s="13" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Shareable one-pager token link + generator not built (frontend of U7-01.39).</t>
+        </is>
+      </c>
       <c r="L26" s="13" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3602,11 +3671,15 @@
       </c>
       <c r="I27" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J27" s="16" t="inlineStr"/>
-      <c r="K27" s="16" t="inlineStr"/>
+      <c r="K27" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: Landing hero one-liner 'Speak the decision. We run the company.' + indigo accent (Landing.js:50-57).</t>
+        </is>
+      </c>
       <c r="L27" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3658,7 +3731,11 @@
         </is>
       </c>
       <c r="J28" s="18" t="inlineStr"/>
-      <c r="K28" s="18" t="inlineStr"/>
+      <c r="K28" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Login errors are raw backend detail passthrough; no actionable copy/'Reset it?' link.</t>
+        </is>
+      </c>
       <c r="L28" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3706,11 +3783,15 @@
       </c>
       <c r="I29" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="J29" s="16" t="inlineStr"/>
-      <c r="K29" s="16" t="inlineStr"/>
+      <c r="K29" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DROP: Obsolete: two-step company+role signup wizard removed; roles now AI-generated from interview (Signup.js PHASES).</t>
+        </is>
+      </c>
       <c r="L29" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3758,11 +3839,15 @@
       </c>
       <c r="I30" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J30" s="18" t="inlineStr"/>
-      <c r="K30" s="18" t="inlineStr"/>
+      <c r="K30" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: Focus rings via --focus-ring both themes; form tab order Email-&gt;Password-&gt;Submit; Enter submits (Login.js:228, index.css:520).</t>
+        </is>
+      </c>
       <c r="L30" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3814,7 +3899,11 @@
         </is>
       </c>
       <c r="J31" s="16" t="inlineStr"/>
-      <c r="K31" s="16" t="inlineStr"/>
+      <c r="K31" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Indigo accent/CTA adopted, but hardcoded neutrals (#16161a/#f7f5f2) + font-black type ramp remain on Landing.</t>
+        </is>
+      </c>
       <c r="L31" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3866,7 +3955,11 @@
         </is>
       </c>
       <c r="J32" s="18" t="inlineStr"/>
-      <c r="K32" s="18" t="inlineStr"/>
+      <c r="K32" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No bottom-anchored/sticky primary CTA + no iOS safe-area handling on auth.</t>
+        </is>
+      </c>
       <c r="L32" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3914,11 +4007,15 @@
       </c>
       <c r="I33" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J33" s="16" t="inlineStr"/>
-      <c r="K33" s="16" t="inlineStr"/>
+      <c r="K33" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: Persistent 4-phase progress bar (signup-phase-bar, Signup.js:54-61).</t>
+        </is>
+      </c>
       <c r="L33" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -3966,11 +4063,15 @@
       </c>
       <c r="I34" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J34" s="18" t="inlineStr"/>
-      <c r="K34" s="18" t="inlineStr"/>
+      <c r="K34" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: WebsiteIntel rotating step captions + scanner, no spinner-in-void (WebsiteIntel.js:8-14).</t>
+        </is>
+      </c>
       <c r="L34" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4022,7 +4123,11 @@
         </is>
       </c>
       <c r="J35" s="16" t="inlineStr"/>
-      <c r="K35" s="16" t="inlineStr"/>
+      <c r="K35" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Conversational one-answer-per-turn frame shipped; actual question wording is backend-generated (VoiceInterview).</t>
+        </is>
+      </c>
       <c r="L35" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4070,11 +4175,15 @@
       </c>
       <c r="I36" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J36" s="18" t="inlineStr"/>
-      <c r="K36" s="18" t="inlineStr"/>
+      <c r="K36" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: BuildReveal staggered framer-motion unveil of count tiles + workflow chips (BuildReveal.js:340-357).</t>
+        </is>
+      </c>
       <c r="L36" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4126,7 +4235,11 @@
         </is>
       </c>
       <c r="J37" s="16" t="inlineStr"/>
-      <c r="K37" s="16" t="inlineStr"/>
+      <c r="K37" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No post-onboarding AI-status banner, no /api/tenant/ai-setup/retry wiring (0 grep hits).</t>
+        </is>
+      </c>
       <c r="L37" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4178,7 +4291,11 @@
         </is>
       </c>
       <c r="J38" s="18" t="inlineStr"/>
-      <c r="K38" s="18" t="inlineStr"/>
+      <c r="K38" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No extracted OnboardingLayout w/ shared H1/subhead/CTA slots; interview type ramp diverges.</t>
+        </is>
+      </c>
       <c r="L38" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4230,7 +4347,11 @@
         </is>
       </c>
       <c r="J39" s="16" t="inlineStr"/>
-      <c r="K39" s="16" t="inlineStr"/>
+      <c r="K39" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Mobile onboarding walkthrough (iPhone SE/Pixel) not done - QA task.</t>
+        </is>
+      </c>
       <c r="L39" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4282,7 +4403,11 @@
         </is>
       </c>
       <c r="J40" s="18" t="inlineStr"/>
-      <c r="K40" s="18" t="inlineStr"/>
+      <c r="K40" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Desk narrative is a deterministic ranker (InsightWell), not LLM; LLM shape deferred to E3-06.</t>
+        </is>
+      </c>
       <c r="L40" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4330,11 +4455,15 @@
       </c>
       <c r="I41" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="J41" s="16" t="inlineStr"/>
-      <c r="K41" s="16" t="inlineStr"/>
+      <c r="K41" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DROP: Obsolete: Desk chip/filter row removed in KR-8, replaced by DecisionBento (sections sized by priority, no filter pills).</t>
+        </is>
+      </c>
       <c r="L41" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4386,7 +4515,11 @@
         </is>
       </c>
       <c r="J42" s="18" t="inlineStr"/>
-      <c r="K42" s="18" t="inlineStr"/>
+      <c r="K42" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Trends deep-links carry filter params; target-screen active-chip-on-arrival still unverified.</t>
+        </is>
+      </c>
       <c r="L42" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4438,7 +4571,11 @@
         </is>
       </c>
       <c r="J43" s="16" t="inlineStr"/>
-      <c r="K43" s="16" t="inlineStr"/>
+      <c r="K43" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Per-section empty copy calmer, but no coaching CTA (capture moved off Desk).</t>
+        </is>
+      </c>
       <c r="L43" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4490,7 +4627,11 @@
         </is>
       </c>
       <c r="J44" s="18" t="inlineStr"/>
-      <c r="K44" s="18" t="inlineStr"/>
+      <c r="K44" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Mobile has always-on DexFab quick-capture; desktop Desk has none (moved to /brain). Desktop muscle-memory gap open.</t>
+        </is>
+      </c>
       <c r="L44" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4542,7 +4683,11 @@
         </is>
       </c>
       <c r="J45" s="16" t="inlineStr"/>
-      <c r="K45" s="16" t="inlineStr"/>
+      <c r="K45" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Section count badges visual-only, no explicit aria-label.</t>
+        </is>
+      </c>
       <c r="L45" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4930,7 +5075,11 @@
         </is>
       </c>
       <c r="J52" s="18" t="inlineStr"/>
-      <c r="K52" s="18" t="inlineStr"/>
+      <c r="K52" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: KR-11 tightened spacing/glass well, but cards intentionally neumorphic (soft shadow), not flattened.</t>
+        </is>
+      </c>
       <c r="L52" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -4982,7 +5131,11 @@
         </is>
       </c>
       <c r="J53" s="16" t="inlineStr"/>
-      <c r="K53" s="16" t="inlineStr"/>
+      <c r="K53" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Tasks capped at 4 w/ '+N more'; no per-card collapse/expand + localStorage memory.</t>
+        </is>
+      </c>
       <c r="L53" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5034,7 +5187,11 @@
         </is>
       </c>
       <c r="J54" s="18" t="inlineStr"/>
-      <c r="K54" s="18" t="inlineStr"/>
+      <c r="K54" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Reason dialog spartan; no char counter, prior-reasons dropdown, role suggestions.</t>
+        </is>
+      </c>
       <c r="L54" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5082,11 +5239,15 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="J55" s="16" t="inlineStr"/>
-      <c r="K55" s="16" t="inlineStr"/>
+      <c r="K55" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DROP: Decision settled: redesign committed to board-only kanban w/ drag-drop; no list view. Record as permanent.</t>
+        </is>
+      </c>
       <c r="L55" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5134,11 +5295,15 @@
       </c>
       <c r="I56" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J56" s="18" t="inlineStr"/>
-      <c r="K56" s="18" t="inlineStr"/>
+      <c r="K56" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: Workflow labels from tenant.operating_model.pipelines[].label; lexicon.workflows retired (Workflows.js:327).</t>
+        </is>
+      </c>
       <c r="L56" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5190,7 +5355,11 @@
         </is>
       </c>
       <c r="J57" s="16" t="inlineStr"/>
-      <c r="K57" s="16" t="inlineStr"/>
+      <c r="K57" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Stages advance via keyboard-operable Advance button; M+arrow keyboard-drag gesture not built.</t>
+        </is>
+      </c>
       <c r="L57" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5238,11 +5407,15 @@
       </c>
       <c r="I58" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="J58" s="18" t="inlineStr"/>
-      <c r="K58" s="18" t="inlineStr"/>
+      <c r="K58" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DROP: Done differently: Contacts merged into single CRM nav; /contacts redirects to /crm (Layout.js:63, App.js:133).</t>
+        </is>
+      </c>
       <c r="L58" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5350,7 +5523,11 @@
         </is>
       </c>
       <c r="J60" s="18" t="inlineStr"/>
-      <c r="K60" s="18" t="inlineStr"/>
+      <c r="K60" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: CSV lands in editable review panel (fix-before-file); no per-row failure/error surfacing on partial import.</t>
+        </is>
+      </c>
       <c r="L60" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5398,11 +5575,15 @@
       </c>
       <c r="I61" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J61" s="16" t="inlineStr"/>
-      <c r="K61" s="16" t="inlineStr"/>
+      <c r="K61" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: Relationship score shows reason sentence + signal chips, desktop + mobile (ContactProfile.js:280-287).</t>
+        </is>
+      </c>
       <c r="L61" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5510,7 +5691,11 @@
         </is>
       </c>
       <c r="J63" s="16" t="inlineStr"/>
-      <c r="K63" s="16" t="inlineStr"/>
+      <c r="K63" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: CRM list/filters at parity on responsive tree; mobile profile AI intel read-only (no rescore/'Score with AI').</t>
+        </is>
+      </c>
       <c r="L63" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5562,7 +5747,11 @@
         </is>
       </c>
       <c r="J64" s="18" t="inlineStr"/>
-      <c r="K64" s="18" t="inlineStr"/>
+      <c r="K64" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Revenue overdue callout shipped; Finance Overview still six equal-weight KPI tiles, no hero metric elevated (Ledger.js:542).</t>
+        </is>
+      </c>
       <c r="L64" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5614,7 +5803,11 @@
         </is>
       </c>
       <c r="J65" s="16" t="inlineStr"/>
-      <c r="K65" s="16" t="inlineStr"/>
+      <c r="K65" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Insight cards have inline 'Ask AI' chip; not the context-routing 'Ask Dex about this' chip (E3-01).</t>
+        </is>
+      </c>
       <c r="L65" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5666,7 +5859,11 @@
         </is>
       </c>
       <c r="J66" s="18" t="inlineStr"/>
-      <c r="K66" s="18" t="inlineStr"/>
+      <c r="K66" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: ReviewPanel not restructured; still on pre-rebrand tokens (brand-600/card-brutal) - only file untouched by karma.</t>
+        </is>
+      </c>
       <c r="L66" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5718,7 +5915,11 @@
         </is>
       </c>
       <c r="J67" s="16" t="inlineStr"/>
-      <c r="K67" s="16" t="inlineStr"/>
+      <c r="K67" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: WhatsAppCard has generic forwarding one-liner; no reply-to-nudge explanation + example.</t>
+        </is>
+      </c>
       <c r="L67" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5770,7 +5971,11 @@
         </is>
       </c>
       <c r="J68" s="18" t="inlineStr"/>
-      <c r="K68" s="18" t="inlineStr"/>
+      <c r="K68" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Expenses flat table; no inline drawer revealing line items.</t>
+        </is>
+      </c>
       <c r="L68" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5818,11 +6023,15 @@
       </c>
       <c r="I69" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="J69" s="16" t="inlineStr"/>
-      <c r="K69" s="16" t="inlineStr"/>
+      <c r="K69" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DROP: Obsolete: FinanceMobile.jsx deleted in KR-10, unified responsive Ledger tree; camera receipt-scan present (Ledger.js:1170).</t>
+        </is>
+      </c>
       <c r="L69" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5874,7 +6083,11 @@
         </is>
       </c>
       <c r="J70" s="18" t="inlineStr"/>
-      <c r="K70" s="18" t="inlineStr"/>
+      <c r="K70" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: DexBadge persona chip on /ask answers only; not an avatar, absent from WorkCoach/OperatingScore narratives.</t>
+        </is>
+      </c>
       <c r="L70" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5926,7 +6139,11 @@
         </is>
       </c>
       <c r="J71" s="16" t="inlineStr"/>
-      <c r="K71" s="16" t="inlineStr"/>
+      <c r="K71" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Dex answers don't stream (blocking); no Stop-generating/retry/copy controls.</t>
+        </is>
+      </c>
       <c r="L71" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -5978,7 +6195,11 @@
         </is>
       </c>
       <c r="J72" s="18" t="inlineStr"/>
-      <c r="K72" s="18" t="inlineStr"/>
+      <c r="K72" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: BrainDocuments search + kind filter shipped; preview-on-hover + 'ask Dex about doc' still missing.</t>
+        </is>
+      </c>
       <c r="L72" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6030,7 +6251,11 @@
         </is>
       </c>
       <c r="J73" s="16" t="inlineStr"/>
-      <c r="K73" s="16" t="inlineStr"/>
+      <c r="K73" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Dex empty state shows example prompts, but static/generic, not industry-specific from operating_model.</t>
+        </is>
+      </c>
       <c r="L73" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6082,7 +6307,11 @@
         </is>
       </c>
       <c r="J74" s="18" t="inlineStr"/>
-      <c r="K74" s="18" t="inlineStr"/>
+      <c r="K74" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No ?context= URL param handling, no pinned/clearable context chip.</t>
+        </is>
+      </c>
       <c r="L74" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6134,7 +6363,11 @@
         </is>
       </c>
       <c r="J75" s="16" t="inlineStr"/>
-      <c r="K75" s="16" t="inlineStr"/>
+      <c r="K75" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No aria-live region on transcript preview; recording announces nothing to SR.</t>
+        </is>
+      </c>
       <c r="L75" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6242,7 +6475,11 @@
         </is>
       </c>
       <c r="J77" s="16" t="inlineStr"/>
-      <c r="K77" s="16" t="inlineStr"/>
+      <c r="K77" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: WorkCoach improvements are text-only; no per-item coach/'working on' affordance.</t>
+        </is>
+      </c>
       <c r="L77" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6294,7 +6531,11 @@
         </is>
       </c>
       <c r="J78" s="18" t="inlineStr"/>
-      <c r="K78" s="18" t="inlineStr"/>
+      <c r="K78" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Roster group headers use tenant role labels; member profile dialog still prints raw role key (Team.js:520).</t>
+        </is>
+      </c>
       <c r="L78" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6346,7 +6587,11 @@
         </is>
       </c>
       <c r="J79" s="16" t="inlineStr"/>
-      <c r="K79" s="16" t="inlineStr"/>
+      <c r="K79" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No shared ContactChip component; person card only reuses kr-bento primitive.</t>
+        </is>
+      </c>
       <c r="L79" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6394,11 +6639,15 @@
       </c>
       <c r="I80" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Dropped</t>
         </is>
       </c>
       <c r="J80" s="18" t="inlineStr"/>
-      <c r="K80" s="18" t="inlineStr"/>
+      <c r="K80" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DROP: Obsolete: no TeamMobile.jsx; redesign made Team.js responsive single-file; role edit in shared MemberDialog.</t>
+        </is>
+      </c>
       <c r="L80" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6450,7 +6699,11 @@
         </is>
       </c>
       <c r="J81" s="16" t="inlineStr"/>
-      <c r="K81" s="16" t="inlineStr"/>
+      <c r="K81" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Notifications flat list; no collapse-by-source + per-group unread (read-state persistence already works).</t>
+        </is>
+      </c>
       <c r="L81" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6502,7 +6755,11 @@
         </is>
       </c>
       <c r="J82" s="18" t="inlineStr"/>
-      <c r="K82" s="18" t="inlineStr"/>
+      <c r="K82" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No weekend zebra/muted-past; past days currently highlighted (opposite).</t>
+        </is>
+      </c>
       <c r="L82" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6554,7 +6811,11 @@
         </is>
       </c>
       <c r="J83" s="16" t="inlineStr"/>
-      <c r="K83" s="16" t="inlineStr"/>
+      <c r="K83" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Leave request streamlined w/ validation+toast; two date inputs (no range picker), explicit Submit (no auto-submit).</t>
+        </is>
+      </c>
       <c r="L83" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6606,7 +6867,11 @@
         </is>
       </c>
       <c r="J84" s="18" t="inlineStr"/>
-      <c r="K84" s="18" t="inlineStr"/>
+      <c r="K84" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Journal decision entries title+chips only; no first-line content preview.</t>
+        </is>
+      </c>
       <c r="L84" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6658,7 +6923,11 @@
         </is>
       </c>
       <c r="J85" s="16" t="inlineStr"/>
-      <c r="K85" s="16" t="inlineStr"/>
+      <c r="K85" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Notif bell synced badge + click-opens-panel + aria-label done; no auto-mark-read behavior.</t>
+        </is>
+      </c>
       <c r="L85" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6710,7 +6979,11 @@
         </is>
       </c>
       <c r="J86" s="18" t="inlineStr"/>
-      <c r="K86" s="18" t="inlineStr"/>
+      <c r="K86" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No Meetings recording surface; mic failure shows generic toast, no settings fallback.</t>
+        </is>
+      </c>
       <c r="L86" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6762,7 +7035,11 @@
         </is>
       </c>
       <c r="J87" s="16" t="inlineStr"/>
-      <c r="K87" s="16" t="inlineStr"/>
+      <c r="K87" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Lexicon editor exists (BusinessVocabulary) but no live-preview panel.</t>
+        </is>
+      </c>
       <c r="L87" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6814,7 +7091,11 @@
         </is>
       </c>
       <c r="J88" s="18" t="inlineStr"/>
-      <c r="K88" s="18" t="inlineStr"/>
+      <c r="K88" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: OperatingModel side-effect param editor not built; only kind chips + delete.</t>
+        </is>
+      </c>
       <c r="L88" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6866,7 +7147,11 @@
         </is>
       </c>
       <c r="J89" s="16" t="inlineStr"/>
-      <c r="K89" s="16" t="inlineStr"/>
+      <c r="K89" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Each settings section has Save button + toast; no per-section dirty/saved-state indicator.</t>
+        </is>
+      </c>
       <c r="L89" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6918,7 +7203,11 @@
         </is>
       </c>
       <c r="J90" s="18" t="inlineStr"/>
-      <c r="K90" s="18" t="inlineStr"/>
+      <c r="K90" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No 2FA/session UI to write copy for; feature absent in Account tab (premise stale).</t>
+        </is>
+      </c>
       <c r="L90" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -6970,7 +7259,11 @@
         </is>
       </c>
       <c r="J91" s="16" t="inlineStr"/>
-      <c r="K91" s="16" t="inlineStr"/>
+      <c r="K91" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Settings forms mix label-above vs inline; no single enforced pattern.</t>
+        </is>
+      </c>
       <c r="L91" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7022,7 +7315,11 @@
         </is>
       </c>
       <c r="J92" s="18" t="inlineStr"/>
-      <c r="K92" s="18" t="inlineStr"/>
+      <c r="K92" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No SettingsMobile.jsx (now responsive Settings.js); 4-tab mobile render/save audit pending.</t>
+        </is>
+      </c>
       <c r="L92" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7074,7 +7371,11 @@
         </is>
       </c>
       <c r="J93" s="16" t="inlineStr"/>
-      <c r="K93" s="16" t="inlineStr"/>
+      <c r="K93" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Admin overview already a metrics dashboard (8 tiles); lacks specific hero metrics (active-this-week, usage-$, tickets).</t>
+        </is>
+      </c>
       <c r="L93" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7126,7 +7427,11 @@
         </is>
       </c>
       <c r="J94" s="18" t="inlineStr"/>
-      <c r="K94" s="18" t="inlineStr"/>
+      <c r="K94" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Admin tenant list flat table; no search/filter/bulk-select.</t>
+        </is>
+      </c>
       <c r="L94" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7178,7 +7483,11 @@
         </is>
       </c>
       <c r="J95" s="16" t="inlineStr"/>
-      <c r="K95" s="16" t="inlineStr"/>
+      <c r="K95" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Per-tenant + per-provider cost present as table+grid; no expand-row, AI-only (no SMS/storage split).</t>
+        </is>
+      </c>
       <c r="L95" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7230,7 +7539,11 @@
         </is>
       </c>
       <c r="J96" s="18" t="inlineStr"/>
-      <c r="K96" s="18" t="inlineStr"/>
+      <c r="K96" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Delete-tenant confirm names blast radius + type-to-confirm; suspend/reset-access/AI-key save still unguarded.</t>
+        </is>
+      </c>
       <c r="L96" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7282,7 +7595,11 @@
         </is>
       </c>
       <c r="J97" s="16" t="inlineStr"/>
-      <c r="K97" s="16" t="inlineStr"/>
+      <c r="K97" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No keyboard-driven bulk actions in admin (depends on 13.2).</t>
+        </is>
+      </c>
       <c r="L97" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7334,7 +7651,11 @@
         </is>
       </c>
       <c r="J98" s="18" t="inlineStr"/>
-      <c r="K98" s="18" t="inlineStr"/>
+      <c r="K98" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Full CSS-var token system live + 0 hardcoded shadows; ~90 hardcoded hex remain (mostly admin/* + Landing).</t>
+        </is>
+      </c>
       <c r="L98" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7386,7 +7707,11 @@
         </is>
       </c>
       <c r="J99" s="16" t="inlineStr"/>
-      <c r="K99" s="16" t="inlineStr"/>
+      <c r="K99" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Fonts unified to one family; no documented H1..caption size scale, 114 arbitrary text-[px] across 27 files.</t>
+        </is>
+      </c>
       <c r="L99" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7438,7 +7763,11 @@
         </is>
       </c>
       <c r="J100" s="18" t="inlineStr"/>
-      <c r="K100" s="18" t="inlineStr"/>
+      <c r="K100" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Default grid is 4pt-aligned but no --space-* token scale or enforcement/audit.</t>
+        </is>
+      </c>
       <c r="L100" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7490,7 +7819,11 @@
         </is>
       </c>
       <c r="J101" s="16" t="inlineStr"/>
-      <c r="K101" s="16" t="inlineStr"/>
+      <c r="K101" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: App largely on @phosphor-icons (74 files); lucide persists in vendored shadcn ui/ primitives; emoji not swept.</t>
+        </is>
+      </c>
       <c r="L101" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7542,7 +7875,11 @@
         </is>
       </c>
       <c r="J102" s="18" t="inlineStr"/>
-      <c r="K102" s="18" t="inlineStr"/>
+      <c r="K102" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: DesignLab + MobileKitchenSink dev harnesses exist; no formal colors/type/spacing/do-don't docs page.</t>
+        </is>
+      </c>
       <c r="L102" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7594,7 +7931,11 @@
         </is>
       </c>
       <c r="J103" s="16" t="inlineStr"/>
-      <c r="K103" s="16" t="inlineStr"/>
+      <c r="K103" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Shared EmptyState in 16 pages/42 usages; not universal (Team/People/Tasks/Workflows thin).</t>
+        </is>
+      </c>
       <c r="L103" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7646,7 +7987,11 @@
         </is>
       </c>
       <c r="J104" s="18" t="inlineStr"/>
-      <c r="K104" s="18" t="inlineStr"/>
+      <c r="K104" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Shaped skeletons on key pages (13 files); animate-spin still in ~17 files.</t>
+        </is>
+      </c>
       <c r="L104" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7698,7 +8043,11 @@
         </is>
       </c>
       <c r="J105" s="16" t="inlineStr"/>
-      <c r="K105" s="16" t="inlineStr"/>
+      <c r="K105" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Retry/plain-language error copy across 19 files; no universal error component, coverage inconsistent.</t>
+        </is>
+      </c>
       <c r="L105" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7750,7 +8099,11 @@
         </is>
       </c>
       <c r="J106" s="18" t="inlineStr"/>
-      <c r="K106" s="18" t="inlineStr"/>
+      <c r="K106" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Some contextual loading copy; generic 'Loading' still in 24 files, not systematically replaced.</t>
+        </is>
+      </c>
       <c r="L106" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7802,7 +8155,11 @@
         </is>
       </c>
       <c r="J107" s="16" t="inlineStr"/>
-      <c r="K107" s="16" t="inlineStr"/>
+      <c r="K107" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Automated UX audit harness exists but no axe-core/Lighthouse contrast pass.</t>
+        </is>
+      </c>
       <c r="L107" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7854,7 +8211,11 @@
         </is>
       </c>
       <c r="J108" s="18" t="inlineStr"/>
-      <c r="K108" s="18" t="inlineStr"/>
+      <c r="K108" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Native tab order OK; custom widgets (kanban) still lack keyboard equivalents.</t>
+        </is>
+      </c>
       <c r="L108" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7902,11 +8263,15 @@
       </c>
       <c r="I109" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J109" s="16" t="inlineStr"/>
-      <c r="K109" s="16" t="inlineStr"/>
+      <c r="K109" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: Single --focus-ring token both themes + global :focus-visible outline (index.css:520,681).</t>
+        </is>
+      </c>
       <c r="L109" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -7958,7 +8323,11 @@
         </is>
       </c>
       <c r="J110" s="18" t="inlineStr"/>
-      <c r="K110" s="18" t="inlineStr"/>
+      <c r="K110" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: aria-label 67 hits/28 files + live regions for toasts/skeletons; icon-only buttons not fully labeled, 2 leaked strings.</t>
+        </is>
+      </c>
       <c r="L110" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8010,7 +8379,11 @@
         </is>
       </c>
       <c r="J111" s="16" t="inlineStr"/>
-      <c r="K111" s="16" t="inlineStr"/>
+      <c r="K111" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Touch-size tokens (44/48/56) + audit rule in place; baseline still flagged many 40x40 controls; current unverified.</t>
+        </is>
+      </c>
       <c r="L111" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8058,11 +8431,15 @@
       </c>
       <c r="I112" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J112" s="18" t="inlineStr"/>
-      <c r="K112" s="18" t="inlineStr"/>
+      <c r="K112" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: prefers-reduced-motion in 7 CSS blocks + JS matchMedia guards (useReveal, Layout, CountUp).</t>
+        </is>
+      </c>
       <c r="L112" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8114,7 +8491,11 @@
         </is>
       </c>
       <c r="J113" s="16" t="inlineStr"/>
-      <c r="K113" s="16" t="inlineStr"/>
+      <c r="K113" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Premise reframed: per-screen *Mobile.jsx obsolete - routes now responsive; remaining work is per-route mobile polish.</t>
+        </is>
+      </c>
       <c r="L113" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8162,11 +8543,15 @@
       </c>
       <c r="I114" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J114" s="18" t="inlineStr"/>
-      <c r="K114" s="18" t="inlineStr"/>
+      <c r="K114" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: InstallPrompt 3rd-session dismissible coach-mark + iOS fallback (InstallPrompt.jsx, Layout.js:534).</t>
+        </is>
+      </c>
       <c r="L114" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8214,11 +8599,15 @@
       </c>
       <c r="I115" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J115" s="16" t="inlineStr"/>
-      <c r="K115" s="16" t="inlineStr"/>
+      <c r="K115" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: Workbox SW NetworkFirst offline caching for read routes + offline.html; money POSTs refuse loudly (service-worker.js).</t>
+        </is>
+      </c>
       <c r="L115" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8266,11 +8655,15 @@
       </c>
       <c r="I116" s="19" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J116" s="18" t="inlineStr"/>
-      <c r="K116" s="18" t="inlineStr"/>
+      <c r="K116" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] DONE: manifest indigo theme + 192/512 maskable icon set (manifest.json).</t>
+        </is>
+      </c>
       <c r="L116" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8322,7 +8715,11 @@
         </is>
       </c>
       <c r="J117" s="16" t="inlineStr"/>
-      <c r="K117" s="16" t="inlineStr"/>
+      <c r="K117" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Some gestures have button equivalents (UndoSnackbar/BottomSheet); no comprehensive switch-control/keyboard parity pass.</t>
+        </is>
+      </c>
       <c r="L117" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8374,7 +8771,11 @@
         </is>
       </c>
       <c r="J118" s="18" t="inlineStr"/>
-      <c r="K118" s="18" t="inlineStr"/>
+      <c r="K118" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Mostly i18n action-verb labels; 1 literal 'Submit' + widespread uppercase labels remain.</t>
+        </is>
+      </c>
       <c r="L118" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8426,7 +8827,11 @@
         </is>
       </c>
       <c r="J119" s="16" t="inlineStr"/>
-      <c r="K119" s="16" t="inlineStr"/>
+      <c r="K119" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: No systematic top-20 error-message rewrite; raw system strings still leak (audit: 2 violations).</t>
+        </is>
+      </c>
       <c r="L119" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8478,7 +8883,11 @@
         </is>
       </c>
       <c r="J120" s="18" t="inlineStr"/>
-      <c r="K120" s="18" t="inlineStr"/>
+      <c r="K120" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Onboarding/Dex/WorkCoach voice consistency - copy audit, no artifact indicating done.</t>
+        </is>
+      </c>
       <c r="L120" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8530,7 +8939,11 @@
         </is>
       </c>
       <c r="J121" s="16" t="inlineStr"/>
-      <c r="K121" s="16" t="inlineStr"/>
+      <c r="K121" s="16" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] PARTIAL: Confirm/Cancel/Discard vocab partly centralized in i18n but used ad-hoc across 24 files; no enforced pairing.</t>
+        </is>
+      </c>
       <c r="L121" s="16" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8582,7 +8995,11 @@
         </is>
       </c>
       <c r="J122" s="18" t="inlineStr"/>
-      <c r="K122" s="18" t="inlineStr"/>
+      <c r="K122" s="18" t="inlineStr">
+        <is>
+          <t>[2026-08-20 karma-validation] KEEP: Epic 7 exit-gate E2E (desktop+iPhone SE+Pixel+tablet) not run - QA sign-off pending.</t>
+        </is>
+      </c>
       <c r="L122" s="18" t="inlineStr">
         <is>
           <t>Founder ask 2026-08-17</t>
@@ -8700,7 +9117,8 @@
       </c>
       <c r="K124" s="13" t="inlineStr">
         <is>
-          <t>Wire target: HeroCard sparkline (U7-01.3 shipped as demo).</t>
+          <t>[2026-08-20 karma-validation] KEEP: BACKEND: no operating_score_history collection, no daily cron, no history endpoint.
+Wire target: HeroCard sparkline (U7-01.3 shipped as demo).</t>
         </is>
       </c>
       <c r="L124" s="13" t="inlineStr">
@@ -8760,7 +9178,8 @@
       </c>
       <c r="K125" s="13" t="inlineStr">
         <is>
-          <t>Wire target: HeroCard DeltaChip (U7-01.1 shipped as demo). Also enables per-employee deltas (U7-01.33).</t>
+          <t>[2026-08-20 karma-validation] KEEP: BACKEND: no week-over-week company.delta (needs history).
+Wire target: HeroCard DeltaChip (U7-01.1 shipped as demo). Also enables per-employee deltas (U7-01.33).</t>
         </is>
       </c>
       <c r="L125" s="13" t="inlineStr">
@@ -8820,7 +9239,8 @@
       </c>
       <c r="K126" s="13" t="inlineStr">
         <is>
-          <t>Wire target: CategoryCard drivers (U7-01.4 shipped as demo).</t>
+          <t>[2026-08-20 karma-validation] KEEP: BACKEND: no per-category drivers in payload; real tenants see blank driver rows.
+Wire target: CategoryCard drivers (U7-01.4 shipped as demo).</t>
         </is>
       </c>
       <c r="L126" s="13" t="inlineStr">
@@ -8880,7 +9300,8 @@
       </c>
       <c r="K127" s="13" t="inlineStr">
         <is>
-          <t>Wire target: CategoryDrillModal (U7-01.5..8 shipped as demo).</t>
+          <t>[2026-08-20 karma-validation] KEEP: BACKEND: no /operating-score/drill/{category} endpoint; real tenants get 'not wired' fallback.
+Wire target: CategoryDrillModal (U7-01.5..8 shipped as demo).</t>
         </is>
       </c>
       <c r="L127" s="13" t="inlineStr">
@@ -8940,7 +9361,8 @@
       </c>
       <c r="K128" s="13" t="inlineStr">
         <is>
-          <t>Wire targets: HeroCard narrative (U7-01.1) + DexExplainerCard (U7-01.9). Both shipped with hardcoded demo text.</t>
+          <t>[2026-08-20 karma-validation] KEEP: BACKEND: no /ai/operating-score-explain endpoint; Dex narrative demo-only.
+Wire targets: HeroCard narrative (U7-01.1) + DexExplainerCard (U7-01.9). Both shipped with hardcoded demo text.</t>
         </is>
       </c>
       <c r="L128" s="13" t="inlineStr">
@@ -9000,7 +9422,8 @@
       </c>
       <c r="K129" s="13" t="inlineStr">
         <is>
-          <t>Wire target: SuggestedActions chip row (U7-01.10 shipped as demo).</t>
+          <t>[2026-08-20 karma-validation] PARTIAL: Suggested-action chips now derive from real stats client-side (karmaScore.js:40); not a backend field; 'lift' estimate dropped as dishonest.
+Wire target: SuggestedActions chip row (U7-01.10 shipped as demo).</t>
         </is>
       </c>
       <c r="L129" s="13" t="inlineStr">
@@ -9060,7 +9483,8 @@
       </c>
       <c r="K130" s="13" t="inlineStr">
         <is>
-          <t>Wire target: Leaderboard per-row delta (U7-01.11 shipped as demo).</t>
+          <t>[2026-08-20 karma-validation] KEEP: BACKEND: no per-employee week-over-week delta; leaderboard shows no delta chip.
+Wire target: Leaderboard per-row delta (U7-01.11 shipped as demo).</t>
         </is>
       </c>
       <c r="L130" s="13" t="inlineStr">
@@ -9120,7 +9544,8 @@
       </c>
       <c r="K131" s="13" t="inlineStr">
         <is>
-          <t>Wire target: FormulaExplainer weights editor (U7-01.17 shipped as demo). Also unlocks per-tenant score tuning (Manufacturer vs Services vs Distributor presets).</t>
+          <t>[2026-08-20 karma-validation] KEEP: BACKEND: weights hardcoded, not read from tenant; FormulaExplainer editor local-only.
+Wire target: FormulaExplainer weights editor (U7-01.17 shipped as demo). Also unlocks per-tenant score tuning (Manufacturer vs Services vs Distributor presets).</t>
         </is>
       </c>
       <c r="L131" s="13" t="inlineStr">
@@ -9180,7 +9605,8 @@
       </c>
       <c r="K132" s="13" t="inlineStr">
         <is>
-          <t>Wire target: InlineCapture form (U7-01.15 shipped as demo).</t>
+          <t>[2026-08-20 karma-validation] KEEP: InlineCapture fake-sends; not wired to POST /api/voice-notes.
+Wire target: InlineCapture form (U7-01.15 shipped as demo).</t>
         </is>
       </c>
       <c r="L132" s="13" t="inlineStr">
@@ -9240,7 +9666,8 @@
       </c>
       <c r="K133" s="13" t="inlineStr">
         <is>
-          <t>Companion to U7-01.31 -- ship together to keep cost bounded.</t>
+          <t>[2026-08-20 karma-validation] KEEP: BACKEND: no 15-min per-tenant cache for explain endpoint (moot until 01.31).
+Companion to U7-01.31 -- ship together to keep cost bounded.</t>
         </is>
       </c>
       <c r="L133" s="13" t="inlineStr">
@@ -9300,7 +9727,8 @@
       </c>
       <c r="K134" s="13" t="inlineStr">
         <is>
-          <t>This is the analysis doc's Phase B in one item. Needs founder sign-off on formula shapes before implementation -- open decision #4.</t>
+          <t>[2026-08-20 karma-validation] KEEP: BACKEND: Phase B metric formulas not applied; responsiveness still penalizes overdue. Needs founder sign-off.
+This is the analysis doc's Phase B in one item. Needs founder sign-off on formula shapes before implementation -- open decision #4.</t>
         </is>
       </c>
       <c r="L134" s="13" t="inlineStr">
@@ -9360,7 +9788,8 @@
       </c>
       <c r="K135" s="13" t="inlineStr">
         <is>
-          <t>Wire target: U7-01.24 (frontend for the setting toggle + email template). Requires an email provider chosen and quota tracked.</t>
+          <t>[2026-08-20 karma-validation] KEEP: BACKEND: no weekly owner digest email cron/template.
+Wire target: U7-01.24 (frontend for the setting toggle + email template). Requires an email provider chosen and quota tracked.</t>
         </is>
       </c>
       <c r="L135" s="13" t="inlineStr">
@@ -9420,7 +9849,8 @@
       </c>
       <c r="K136" s="13" t="inlineStr">
         <is>
-          <t>Wire target: U7-01.25 (frontend share page + generator UI). Board-of-directors friendly one-pager, no auth needed.</t>
+          <t>[2026-08-20 karma-validation] KEEP: BACKEND: no signed-token public one-pager endpoint.
+Wire target: U7-01.25 (frontend share page + generator UI). Board-of-directors friendly one-pager, no auth needed.</t>
         </is>
       </c>
       <c r="L136" s="13" t="inlineStr">
@@ -10832,7 +11262,8 @@
       <c r="J161" s="16" t="n"/>
       <c r="K161" s="16" t="inlineStr">
         <is>
-          <t>Noted 2026-08-17 during the RD-5 sweep.</t>
+          <t>[2026-08-20 karma-validation] KEEP: Admin portal confirmed still on legacy theme (deliberate deferral).
+Noted 2026-08-17 during the RD-5 sweep.</t>
         </is>
       </c>
       <c r="L161" s="16" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): log the 20 karma-mobile commits into Epic 7
Karma-redesign shipped 20 UI commits between KR-14.1 (2026-08-19) and
KM-16 (2026-08-27) — the desktop bento cleanup plus the KR-14.2-24 /
KM-1..16 mobile pass. None of them were recorded in the source Epic 7
xlsx (karma's own tracker commit only bumped the generated dashboard
HTML), so the ledger has been under-reporting Epic 7 by 20 items since
the merge landed in d810145.

Recorded as Sprint 19 = "Karma mobile pass — shipped" (20/20 COMPLETE)
in Epic 7's Backlog + Dashboard, with a per-commit trail also added to
the "UI Redesign Log" sheet (r86..r105). The Dashboard "Redesign log"
counter was left at 21/22 so the same 20 commits aren't counted twice —
Sprint 19 carries the total. Master Tracker Epic 7 -> 105/195 (was
64/153), all-epics banner -> 494/648, ledger HTML regenerated.

No code changes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
+++ b/docs/DecisionOS_Epic7_UX_UI_Optimization.xlsx
@@ -1464,7 +1464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1497,6 +1497,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
@@ -2131,33 +2132,66 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Sprint 19</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>20</v>
+      </c>
+      <c r="D24" t="n">
+        <v>20</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>20 UI commits from karma-redesign (KR-14.2 desktop cleanup + KR-14.2-24 and KM-1..16 mobile pass). Every commit shipped to Backend_optimization via merge d810145 (2026-08-28).</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Redesign log</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>KR/RD redesign changelog (shipped during rebuild)</t>
         </is>
       </c>
-      <c r="C24" t="n">
+      <c r="C25" t="n">
         <v>21</v>
       </c>
-      <c r="D24" t="n">
+      <c r="D25" t="n">
         <v>22</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>95%</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>In progress</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>See 'UI Redesign Log' sheet — 81 karma/RD/NM/MPWA UI commits, all shipped to Backend_optimization.</t>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>See 'UI Redesign Log' sheet — 105 karma / RD / NM / MPWA UI commits, all shipped to Backend_optimization. Sprint 19 carries the KM-* / KR-14.2-24 mobile pass entries in Backlog to keep the totals clean.</t>
         </is>
       </c>
     </row>
@@ -2172,7 +2206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4410,6 +4444,546 @@
         </is>
       </c>
     </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Karma (final design language — shipped)</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>bb1365c</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="D86" s="7" t="inlineStr">
+        <is>
+          <t>KR-14.2 — the bento loses its fog and its dead air</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>a0b472c</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>KM-1 — mobile pass 1: /inbox reflow + shared foundation + 7 verified bugs</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>7df035a</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="D88" s="7" t="inlineStr">
+        <is>
+          <t>KR-14.2–14.17 — the phone gets its own layout, the desktop is left alone</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>06947a3</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>KR-14.18–14.24 — mobile pass 2: desk KPI strip, workflow accordions, task expanded body</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>d230bf5</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="D90" s="7" t="inlineStr">
+        <is>
+          <t>KM-3 — mobile pass 3: my-work, calendar, desk band, More panel, Dex voice</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>29cb4ef</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>KM-4 — /finance: all six tabs reachable, five tables become cards on a phone</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>25fe1fe</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D92" s="7" t="inlineStr">
+        <is>
+          <t>KM-5 — inbox card pill, my-work step gestures, calendar-free finance, dock menu</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>7cde42b</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>KM-6 — checklist strip, progress-only status bar, arrows back on step rows</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ca396f4</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D94" s="7" t="inlineStr">
+        <is>
+          <t>KM-7 — overdue pill row, one-row task actions, neumorphic plan editor, dock-width More</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>91a4c7e</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>KM-8 — the More menu goes light: no scrim, minimal glass, seven equal panes</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>5f04a36</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D96" s="7" t="inlineStr">
+        <is>
+          <t>KM-9 — More menu: no close button, fits its content, static tiles, slight dim</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>d780f7f</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>KM-9b — /inbox: progressive blur removed, band pulled clear of the dock</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>b128ee6</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D98" s="7" t="inlineStr">
+        <is>
+          <t>KM-10 — New Task dialog and contact profiles onto the neumorphic system</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>67b71c9</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>KM-10b — /journal rebuilt: neumorphic, calendar view + date picking</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>0e08e2d</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="inlineStr">
+        <is>
+          <t>KM-11 — Dex moves into the bottom bar: ribbon wave + edge vignette</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>8fd0705</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D101" s="7" t="inlineStr">
+        <is>
+          <t>KM-12 — the decision review dialog joins the design system</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>b7f9441</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D102" s="7" t="inlineStr">
+        <is>
+          <t>KM-13 — /inbox takes the founder's glow artwork as its sky</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>b279883</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D103" s="7" t="inlineStr">
+        <is>
+          <t>KM-14 — the glow artwork is desktop-only; mobile keeps its gradient sky</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>6a34aa6</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D104" s="7" t="inlineStr">
+        <is>
+          <t>KM-15 — mobile /inbox takes the new glow artwork as a 9 KB WebP</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Karma mobile pass — shipped</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>b8f72a5</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+      <c r="D105" s="7" t="inlineStr">
+        <is>
+          <t>KM-16 — nudge the mobile glow so the grey core clears the greeting</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4421,7 +4995,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L154"/>
+  <dimension ref="A1:L174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -13150,13 +13724,1126 @@
         </is>
       </c>
     </row>
-    <row r="155" ht="70" customHeight="1"/>
-    <row r="156" ht="70" customHeight="1"/>
-    <row r="157" ht="70" customHeight="1"/>
-    <row r="158" ht="70" customHeight="1"/>
-    <row r="159" ht="70" customHeight="1"/>
-    <row r="160" ht="70" customHeight="1"/>
-    <row r="161" ht="70" customHeight="1"/>
+    <row r="155" ht="70" customHeight="1">
+      <c r="A155" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.1</t>
+        </is>
+      </c>
+      <c r="B155" s="16" t="inlineStr">
+        <is>
+          <t>Desk (bento)</t>
+        </is>
+      </c>
+      <c r="C155" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D155" s="15" t="inlineStr">
+        <is>
+          <t>Karma polish</t>
+        </is>
+      </c>
+      <c r="E155" s="16" t="inlineStr">
+        <is>
+          <t>KR-14.2 · bento loses its fog and its dead air</t>
+        </is>
+      </c>
+      <c r="F155" s="16" t="inlineStr">
+        <is>
+          <t>Desktop bento clarity pass: killed the fog-veil overlay and reclaimed the dead air around the tiles.</t>
+        </is>
+      </c>
+      <c r="G155" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H155" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I155" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J155" s="16" t="n"/>
+      <c r="K155" s="16" t="inlineStr">
+        <is>
+          <t>Commit bb1365c. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L155" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="70" customHeight="1">
+      <c r="A156" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.2</t>
+        </is>
+      </c>
+      <c r="B156" s="16" t="inlineStr">
+        <is>
+          <t>Mobile /inbox</t>
+        </is>
+      </c>
+      <c r="C156" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D156" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E156" s="16" t="inlineStr">
+        <is>
+          <t>KM-1 · mobile pass 1: /inbox reflow + shared foundation</t>
+        </is>
+      </c>
+      <c r="F156" s="16" t="inlineStr">
+        <is>
+          <t>First real mobile pass on /inbox: reflow, shared mobile foundation module, 7 verified bugs squashed.</t>
+        </is>
+      </c>
+      <c r="G156" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H156" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I156" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J156" s="16" t="n"/>
+      <c r="K156" s="16" t="inlineStr">
+        <is>
+          <t>Commit a0b472c. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L156" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="70" customHeight="1">
+      <c r="A157" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.3</t>
+        </is>
+      </c>
+      <c r="B157" s="16" t="inlineStr">
+        <is>
+          <t>Mobile shell (all pages)</t>
+        </is>
+      </c>
+      <c r="C157" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D157" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E157" s="16" t="inlineStr">
+        <is>
+          <t>KR-14.2–14.17 · the phone gets its own layout, the desktop is left alone</t>
+        </is>
+      </c>
+      <c r="F157" s="16" t="inlineStr">
+        <is>
+          <t>16-step mobile layout: dedicated phone layout across the app while the desktop shell stays untouched.</t>
+        </is>
+      </c>
+      <c r="G157" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H157" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I157" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J157" s="16" t="n"/>
+      <c r="K157" s="16" t="inlineStr">
+        <is>
+          <t>Commit 7df035a. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L157" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="70" customHeight="1">
+      <c r="A158" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.4</t>
+        </is>
+      </c>
+      <c r="B158" s="16" t="inlineStr">
+        <is>
+          <t>Mobile /desk, /workflows, /tasks</t>
+        </is>
+      </c>
+      <c r="C158" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D158" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E158" s="16" t="inlineStr">
+        <is>
+          <t>KR-14.18–14.24 · mobile pass 2: desk KPI strip, workflow accordions, task expanded body</t>
+        </is>
+      </c>
+      <c r="F158" s="16" t="inlineStr">
+        <is>
+          <t>Mobile pass 2: mobile desk KPI strip, workflow board becomes accordions, task cards get an expanded body.</t>
+        </is>
+      </c>
+      <c r="G158" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H158" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I158" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J158" s="16" t="n"/>
+      <c r="K158" s="16" t="inlineStr">
+        <is>
+          <t>Commit 06947a3. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L158" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="70" customHeight="1">
+      <c r="A159" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.5</t>
+        </is>
+      </c>
+      <c r="B159" s="16" t="inlineStr">
+        <is>
+          <t>Mobile /my-work, /calendar, dock</t>
+        </is>
+      </c>
+      <c r="C159" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D159" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E159" s="16" t="inlineStr">
+        <is>
+          <t>KM-3 · mobile pass 3: my-work, calendar, desk band, More panel, Dex voice</t>
+        </is>
+      </c>
+      <c r="F159" s="16" t="inlineStr">
+        <is>
+          <t>Third mobile pass: my-work, calendar, desk band, More panel and Dex voice all reflowed.</t>
+        </is>
+      </c>
+      <c r="G159" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H159" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I159" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J159" s="16" t="n"/>
+      <c r="K159" s="16" t="inlineStr">
+        <is>
+          <t>Commit d230bf5. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L159" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="70" customHeight="1">
+      <c r="A160" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.6</t>
+        </is>
+      </c>
+      <c r="B160" s="16" t="inlineStr">
+        <is>
+          <t>Mobile /finance</t>
+        </is>
+      </c>
+      <c r="C160" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D160" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E160" s="16" t="inlineStr">
+        <is>
+          <t>KM-4 · /finance: all six tabs reachable, five tables become cards on a phone</t>
+        </is>
+      </c>
+      <c r="F160" s="16" t="inlineStr">
+        <is>
+          <t>Finance mobile: every one of the six tabs reachable on a phone, five tables rebuilt as card lists.</t>
+        </is>
+      </c>
+      <c r="G160" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H160" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I160" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J160" s="16" t="n"/>
+      <c r="K160" s="16" t="inlineStr">
+        <is>
+          <t>Commit 29cb4ef. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L160" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="70" customHeight="1">
+      <c r="A161" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.7</t>
+        </is>
+      </c>
+      <c r="B161" s="16" t="inlineStr">
+        <is>
+          <t>/inbox card, my-work steps, /finance</t>
+        </is>
+      </c>
+      <c r="C161" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D161" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E161" s="16" t="inlineStr">
+        <is>
+          <t>KM-5 · inbox card pill, my-work step gestures, calendar-free finance, dock menu</t>
+        </is>
+      </c>
+      <c r="F161" s="16" t="inlineStr">
+        <is>
+          <t>Inbox card pill, my-work step gestures, finance without the calendar surface, dock-driven menu.</t>
+        </is>
+      </c>
+      <c r="G161" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H161" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I161" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J161" s="16" t="n"/>
+      <c r="K161" s="16" t="inlineStr">
+        <is>
+          <t>Commit 25fe1fe. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L161" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.8</t>
+        </is>
+      </c>
+      <c r="B162" s="16" t="inlineStr">
+        <is>
+          <t>Task detail, checklist</t>
+        </is>
+      </c>
+      <c r="C162" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D162" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E162" s="16" t="inlineStr">
+        <is>
+          <t>KM-6 · checklist strip, progress-only status bar, arrows back on step rows</t>
+        </is>
+      </c>
+      <c r="F162" s="16" t="inlineStr">
+        <is>
+          <t>Checklist strip added, status bar becomes a progress track, back-arrows restored on step rows.</t>
+        </is>
+      </c>
+      <c r="G162" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H162" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I162" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J162" s="16" t="n"/>
+      <c r="K162" s="16" t="inlineStr">
+        <is>
+          <t>Commit 7cde42b. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L162" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.9</t>
+        </is>
+      </c>
+      <c r="B163" s="16" t="inlineStr">
+        <is>
+          <t>Tasks, plan editor, More menu</t>
+        </is>
+      </c>
+      <c r="C163" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D163" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E163" s="16" t="inlineStr">
+        <is>
+          <t>KM-7 · overdue pill row, one-row task actions, neumorphic plan editor, dock-width More</t>
+        </is>
+      </c>
+      <c r="F163" s="16" t="inlineStr">
+        <is>
+          <t>Overdue pill row, one-row task actions, plan editor rebuilt neumorphic, More menu takes dock width.</t>
+        </is>
+      </c>
+      <c r="G163" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H163" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I163" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J163" s="16" t="n"/>
+      <c r="K163" s="16" t="inlineStr">
+        <is>
+          <t>Commit ca396f4. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L163" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.10</t>
+        </is>
+      </c>
+      <c r="B164" s="16" t="inlineStr">
+        <is>
+          <t>More menu</t>
+        </is>
+      </c>
+      <c r="C164" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D164" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E164" s="16" t="inlineStr">
+        <is>
+          <t>KM-8 · More menu goes light — no scrim, minimal glass, seven equal panes</t>
+        </is>
+      </c>
+      <c r="F164" s="16" t="inlineStr">
+        <is>
+          <t>Light More menu: no scrim, minimal glass, seven equally-weighted panes.</t>
+        </is>
+      </c>
+      <c r="G164" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H164" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I164" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J164" s="16" t="n"/>
+      <c r="K164" s="16" t="inlineStr">
+        <is>
+          <t>Commit 91a4c7e. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L164" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.11</t>
+        </is>
+      </c>
+      <c r="B165" s="16" t="inlineStr">
+        <is>
+          <t>More menu</t>
+        </is>
+      </c>
+      <c r="C165" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D165" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E165" s="16" t="inlineStr">
+        <is>
+          <t>KM-9 · More menu — no close button, fits its content, static tiles, slight dim</t>
+        </is>
+      </c>
+      <c r="F165" s="16" t="inlineStr">
+        <is>
+          <t>More menu polish: close button removed, panel fits its content, tiles static, page dims slightly.</t>
+        </is>
+      </c>
+      <c r="G165" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H165" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I165" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J165" s="16" t="n"/>
+      <c r="K165" s="16" t="inlineStr">
+        <is>
+          <t>Commit 5f04a36. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L165" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.12</t>
+        </is>
+      </c>
+      <c r="B166" s="16" t="inlineStr">
+        <is>
+          <t>/inbox, dock</t>
+        </is>
+      </c>
+      <c r="C166" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D166" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E166" s="16" t="inlineStr">
+        <is>
+          <t>KM-9b · /inbox: progressive blur removed, band pulled clear of the dock</t>
+        </is>
+      </c>
+      <c r="F166" s="16" t="inlineStr">
+        <is>
+          <t>/inbox: killed progressive blur that muddied cards; band pulled clear of the dock overlap.</t>
+        </is>
+      </c>
+      <c r="G166" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H166" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I166" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J166" s="16" t="n"/>
+      <c r="K166" s="16" t="inlineStr">
+        <is>
+          <t>Commit d780f7f. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L166" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.13</t>
+        </is>
+      </c>
+      <c r="B167" s="16" t="inlineStr">
+        <is>
+          <t>New Task dialog, contact profile</t>
+        </is>
+      </c>
+      <c r="C167" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D167" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E167" s="16" t="inlineStr">
+        <is>
+          <t>KM-10 · New Task dialog and contact profiles onto the neumorphic system</t>
+        </is>
+      </c>
+      <c r="F167" s="16" t="inlineStr">
+        <is>
+          <t>New Task dialog and contact profile move onto the shared neumorphic system.</t>
+        </is>
+      </c>
+      <c r="G167" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H167" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I167" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J167" s="16" t="n"/>
+      <c r="K167" s="16" t="inlineStr">
+        <is>
+          <t>Commit b128ee6. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L167" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.14</t>
+        </is>
+      </c>
+      <c r="B168" s="16" t="inlineStr">
+        <is>
+          <t>/journal</t>
+        </is>
+      </c>
+      <c r="C168" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D168" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E168" s="16" t="inlineStr">
+        <is>
+          <t>KM-10b · /journal rebuilt — neumorphic, calendar view + date picking</t>
+        </is>
+      </c>
+      <c r="F168" s="16" t="inlineStr">
+        <is>
+          <t>/journal rebuilt on the neumorphic system with a calendar view and real date picking.</t>
+        </is>
+      </c>
+      <c r="G168" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H168" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I168" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J168" s="16" t="n"/>
+      <c r="K168" s="16" t="inlineStr">
+        <is>
+          <t>Commit 67b71c9. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L168" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.15</t>
+        </is>
+      </c>
+      <c r="B169" s="16" t="inlineStr">
+        <is>
+          <t>Dex bottom-bar</t>
+        </is>
+      </c>
+      <c r="C169" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D169" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E169" s="16" t="inlineStr">
+        <is>
+          <t>KM-11 · Dex moves into the bottom bar: ribbon wave + edge vignette</t>
+        </is>
+      </c>
+      <c r="F169" s="16" t="inlineStr">
+        <is>
+          <t>Dex moves into the bottom bar; adds ribbon-wave listening motion and an edge vignette.</t>
+        </is>
+      </c>
+      <c r="G169" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H169" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I169" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J169" s="16" t="n"/>
+      <c r="K169" s="16" t="inlineStr">
+        <is>
+          <t>Commit 0e08e2d. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L169" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.16</t>
+        </is>
+      </c>
+      <c r="B170" s="16" t="inlineStr">
+        <is>
+          <t>Decision review dialog</t>
+        </is>
+      </c>
+      <c r="C170" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D170" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E170" s="16" t="inlineStr">
+        <is>
+          <t>KM-12 · the decision review dialog joins the design system</t>
+        </is>
+      </c>
+      <c r="F170" s="16" t="inlineStr">
+        <is>
+          <t>The decision review dialog is brought onto the karma design system.</t>
+        </is>
+      </c>
+      <c r="G170" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H170" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I170" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J170" s="16" t="n"/>
+      <c r="K170" s="16" t="inlineStr">
+        <is>
+          <t>Commit 8fd0705. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L170" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.17</t>
+        </is>
+      </c>
+      <c r="B171" s="16" t="inlineStr">
+        <is>
+          <t>/inbox background</t>
+        </is>
+      </c>
+      <c r="C171" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D171" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E171" s="16" t="inlineStr">
+        <is>
+          <t>KM-13 · /inbox takes the founder's glow artwork as its sky</t>
+        </is>
+      </c>
+      <c r="F171" s="16" t="inlineStr">
+        <is>
+          <t>The founder-supplied glow artwork is adopted as /inbox's ambient sky.</t>
+        </is>
+      </c>
+      <c r="G171" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H171" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I171" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J171" s="16" t="n"/>
+      <c r="K171" s="16" t="inlineStr">
+        <is>
+          <t>Commit b7f9441. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L171" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.18</t>
+        </is>
+      </c>
+      <c r="B172" s="16" t="inlineStr">
+        <is>
+          <t>/inbox background (desktop)</t>
+        </is>
+      </c>
+      <c r="C172" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D172" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E172" s="16" t="inlineStr">
+        <is>
+          <t>KM-14 · glow artwork is desktop-only; mobile keeps its gradient sky</t>
+        </is>
+      </c>
+      <c r="F172" s="16" t="inlineStr">
+        <is>
+          <t>Restricted the glow artwork to desktop only; mobile keeps its lighter gradient sky.</t>
+        </is>
+      </c>
+      <c r="G172" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H172" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I172" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J172" s="16" t="n"/>
+      <c r="K172" s="16" t="inlineStr">
+        <is>
+          <t>Commit b279883. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L172" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.19</t>
+        </is>
+      </c>
+      <c r="B173" s="16" t="inlineStr">
+        <is>
+          <t>/inbox mobile background</t>
+        </is>
+      </c>
+      <c r="C173" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D173" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E173" s="16" t="inlineStr">
+        <is>
+          <t>KM-15 · mobile /inbox takes the new glow artwork as a 9 KB WebP</t>
+        </is>
+      </c>
+      <c r="F173" s="16" t="inlineStr">
+        <is>
+          <t>Mobile /inbox takes the new glow artwork shipped as a 9 KB WebP asset.</t>
+        </is>
+      </c>
+      <c r="G173" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H173" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I173" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J173" s="16" t="n"/>
+      <c r="K173" s="16" t="inlineStr">
+        <is>
+          <t>Commit 6a34aa6. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L173" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="16" t="inlineStr">
+        <is>
+          <t>U7-19.20</t>
+        </is>
+      </c>
+      <c r="B174" s="16" t="inlineStr">
+        <is>
+          <t>/inbox mobile background</t>
+        </is>
+      </c>
+      <c r="C174" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="D174" s="15" t="inlineStr">
+        <is>
+          <t>Mobile pass</t>
+        </is>
+      </c>
+      <c r="E174" s="16" t="inlineStr">
+        <is>
+          <t>KM-16 · nudge the mobile glow so the grey core clears the greeting</t>
+        </is>
+      </c>
+      <c r="F174" s="16" t="inlineStr">
+        <is>
+          <t>Nudged the mobile glow so its grey core clears the greeting text underneath.</t>
+        </is>
+      </c>
+      <c r="G174" s="16" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H174" s="16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="I174" s="19" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J174" s="16" t="n"/>
+      <c r="K174" s="16" t="inlineStr">
+        <is>
+          <t>Commit b8f72a5. Landed on karma-redesign, merged into Backend_optimization via d810145.</t>
+        </is>
+      </c>
+      <c r="L174" s="16" t="inlineStr">
+        <is>
+          <t>karma-redesign (Chinmay) — recorded 2026-08-28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>